<commit_message>
updating logic for sample fraction for display in Hows My Waterway
</commit_message>
<xml_diff>
--- a/other/input/wqx_templates/wqx_template_matching_table.xlsx
+++ b/other/input/wqx_templates/wqx_template_matching_table.xlsx
@@ -1,41 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="34776" yWindow="-1980" windowWidth="21600" windowHeight="11292" tabRatio="756" activeTab="1"/>
+    <workbookView xWindow="34776" yWindow="-1980" windowWidth="21600" windowHeight="11292" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="site_coordinates" sheetId="1" r:id="rId1"/>
-    <sheet name="adec_site_names" sheetId="6" r:id="rId2"/>
-    <sheet name="result_sample_fraction" sheetId="2" r:id="rId3"/>
-    <sheet name="result_detection_condition" sheetId="3" r:id="rId4"/>
-    <sheet name="chemical_preservative" sheetId="4" r:id="rId5"/>
-    <sheet name="sample_container_type_color" sheetId="5" r:id="rId6"/>
+    <sheet name="site_coordinates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="adec_site_names" sheetId="6" state="visible" r:id="rId2"/>
+    <sheet name="result_sample_fraction" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="result_detection_condition" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="chemical_preservative" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="sample_container_type_color" sheetId="5" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Author</author>
   </authors>
@@ -50,7 +33,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     List dissolved metals as 'Filtered, field' or 'Filtered, lab'. Total metals will be 'Unfiltered'</t>
@@ -62,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="224">
   <si>
     <t>KR RM 0 NNC</t>
   </si>
@@ -584,13 +567,164 @@
   </si>
   <si>
     <t>KBL_t_44.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">result_sample_fraction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">analytical_method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acid Soluble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bed Sediment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bedload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bioavailable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comb Available</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dissolved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extractable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filterable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dissolved metals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtered, lab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free Available</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inorganic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leachable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-Filterable (Particle)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">non-linear function</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-settleable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-volatile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pot. Dissolved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semivolatile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Settleable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strong Acid Diss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supernate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suspended</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total suspended solids</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2540-D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total nitrate/nitrite-N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SM21 4500NO3-F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total phosphorus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SM21 4500P-B,E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Recoverable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Residual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Soluble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unfiltered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total metals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unfiltered, field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vapor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volatile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BTEX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SW8260D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weak Acid Diss</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -599,12 +733,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <b/>
     </font>
   </fonts>
   <fills count="3">
@@ -630,13 +769,9 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -644,13 +779,13 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -932,16 +1067,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="21.109375" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="21.88671875" customWidth="1"/>
+    <col min="1" max="1" width="21.109375" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="21.88671875" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" t="s">
         <v>48</v>
       </c>
@@ -955,11 +1090,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2">
+    <row r="2">
+      <c r="A2" t="n">
         <v>60.550888</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="n">
         <v>-151.268417</v>
       </c>
       <c r="C2" t="s">
@@ -969,11 +1104,11 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3">
+    <row r="3">
+      <c r="A3" t="n">
         <v>60.543680000000002</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="n">
         <v>-151.22293999999999</v>
       </c>
       <c r="C3" t="s">
@@ -983,11 +1118,11 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4">
+    <row r="4">
+      <c r="A4" t="n">
         <v>60.539279000000001</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="n">
         <v>-151.14226300000001</v>
       </c>
       <c r="C4" t="s">
@@ -997,11 +1132,11 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5">
+    <row r="5">
+      <c r="A5" t="n">
         <v>60.548029</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="n">
         <v>-151.14323999999999</v>
       </c>
       <c r="C5" t="s">
@@ -1011,11 +1146,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6">
+    <row r="6">
+      <c r="A6" t="n">
         <v>60.533743000000001</v>
       </c>
-      <c r="B6">
+      <c r="B6" t="n">
         <v>-151.09925799999999</v>
       </c>
       <c r="C6" t="s">
@@ -1028,11 +1163,11 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7">
+    <row r="7">
+      <c r="A7" t="n">
         <v>60.502004999999997</v>
       </c>
-      <c r="B7">
+      <c r="B7" t="n">
         <v>-151.10697300000001</v>
       </c>
       <c r="C7" t="s">
@@ -1042,11 +1177,11 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8">
+    <row r="8">
+      <c r="A8" t="n">
         <v>60.482317999999999</v>
       </c>
-      <c r="B8">
+      <c r="B8" t="n">
         <v>-151.12705299999999</v>
       </c>
       <c r="C8" t="s">
@@ -1056,11 +1191,11 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9">
+    <row r="9">
+      <c r="A9" t="n">
         <v>60.476633999999997</v>
       </c>
-      <c r="B9">
+      <c r="B9" t="n">
         <v>-151.082099</v>
       </c>
       <c r="C9" t="s">
@@ -1070,11 +1205,11 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10">
+    <row r="10">
+      <c r="A10" t="n">
         <v>60.483364000000002</v>
       </c>
-      <c r="B10">
+      <c r="B10" t="n">
         <v>-151.05765600000001</v>
       </c>
       <c r="C10" t="s">
@@ -1084,11 +1219,11 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11">
+    <row r="11">
+      <c r="A11" t="n">
         <v>60.480338000000003</v>
       </c>
-      <c r="B11">
+      <c r="B11" t="n">
         <v>-151.03084699999999</v>
       </c>
       <c r="C11" t="s">
@@ -1098,11 +1233,11 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12">
+    <row r="12">
+      <c r="A12" t="n">
         <v>60.489963000000003</v>
       </c>
-      <c r="B12">
+      <c r="B12" t="n">
         <v>-150.86098200000001</v>
       </c>
       <c r="C12" t="s">
@@ -1112,11 +1247,11 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13">
+    <row r="13">
+      <c r="A13" t="n">
         <v>60.498283999999998</v>
       </c>
-      <c r="B13">
+      <c r="B13" t="n">
         <v>-150.86312100000001</v>
       </c>
       <c r="C13" t="s">
@@ -1126,11 +1261,11 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14">
+    <row r="14">
+      <c r="A14" t="n">
         <v>60.53687</v>
       </c>
-      <c r="B14">
+      <c r="B14" t="n">
         <v>-150.75472400000001</v>
       </c>
       <c r="C14" t="s">
@@ -1140,11 +1275,11 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15">
+    <row r="15">
+      <c r="A15" t="n">
         <v>60.515441000000003</v>
       </c>
-      <c r="B15">
+      <c r="B15" t="n">
         <v>-150.70206899999999</v>
       </c>
       <c r="C15" t="s">
@@ -1154,8 +1289,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16">
+    <row r="16">
+      <c r="A16" t="n">
         <v>60.489843999999998</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1168,11 +1303,11 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17">
+    <row r="17">
+      <c r="A17" t="n">
         <v>60.481518000000001</v>
       </c>
-      <c r="B17">
+      <c r="B17" t="n">
         <v>-150.632498</v>
       </c>
       <c r="C17" t="s">
@@ -1182,11 +1317,11 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18">
+    <row r="18">
+      <c r="A18" t="n">
         <v>60.467517000000001</v>
       </c>
-      <c r="B18">
+      <c r="B18" t="n">
         <v>-150.507789</v>
       </c>
       <c r="C18" t="s">
@@ -1196,11 +1331,11 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19">
+    <row r="19">
+      <c r="A19" t="n">
         <v>60.54081</v>
       </c>
-      <c r="B19">
+      <c r="B19" t="n">
         <v>-151.18278000000001</v>
       </c>
       <c r="C19" t="s">
@@ -1210,11 +1345,11 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20">
+    <row r="20">
+      <c r="A20" t="n">
         <v>60.481392</v>
       </c>
-      <c r="B20">
+      <c r="B20" t="n">
         <v>-150.11501999999999</v>
       </c>
       <c r="C20" t="s">
@@ -1224,11 +1359,11 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21">
+    <row r="21">
+      <c r="A21" t="n">
         <v>60.484622000000002</v>
       </c>
-      <c r="B21">
+      <c r="B21" t="n">
         <v>-149.993955</v>
       </c>
       <c r="C21" t="s">
@@ -1238,11 +1373,11 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22">
+    <row r="22">
+      <c r="A22" t="n">
         <v>60.488999999999997</v>
       </c>
-      <c r="B22">
+      <c r="B22" t="n">
         <v>-149.87700000000001</v>
       </c>
       <c r="C22" t="s">
@@ -1252,11 +1387,11 @@
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23">
+    <row r="23">
+      <c r="A23" t="n">
         <v>60.492007000000001</v>
       </c>
-      <c r="B23">
+      <c r="B23" t="n">
         <v>-149.810844</v>
       </c>
       <c r="C23" t="s">
@@ -1268,22 +1403,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="21.88671875" customWidth="1"/>
-    <col min="2" max="2" width="34.6640625" customWidth="1"/>
-    <col min="3" max="3" width="25.44140625" customWidth="1"/>
-    <col min="4" max="4" width="25.33203125" customWidth="1"/>
+    <col min="1" max="1" width="21.88671875" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="34.6640625" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="25.44140625" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="25.33203125" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" t="s">
         <v>46</v>
       </c>
@@ -1297,7 +1432,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1311,7 +1446,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -1325,7 +1460,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1339,7 +1474,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1353,7 +1488,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1370,7 +1505,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1384,7 +1519,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -1398,7 +1533,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1412,7 +1547,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -1426,7 +1561,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -1440,7 +1575,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -1454,7 +1589,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -1468,7 +1603,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -1482,7 +1617,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -1496,7 +1631,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -1510,7 +1645,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -1524,7 +1659,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1538,7 +1673,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -1552,7 +1687,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1566,7 +1701,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -1580,7 +1715,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22">
       <c r="A22" t="s">
         <v>38</v>
       </c>
@@ -1594,7 +1729,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23">
       <c r="A23" t="s">
         <v>40</v>
       </c>
@@ -1610,266 +1745,329 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C38"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="27.44140625" customWidth="1"/>
-    <col min="2" max="2" width="25.44140625" customWidth="1"/>
+    <col min="1" max="1" width="27.44140625" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="25.44140625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" s="2" t="s">
-        <v>94</v>
+        <v>174</v>
       </c>
       <c r="B1" t="s">
-        <v>89</v>
+        <v>175</v>
       </c>
       <c r="C1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>177</v>
+      </c>
+      <c r="B2"/>
+      <c r="C2"/>
+    </row>
+    <row r="3">
       <c r="A3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>178</v>
+      </c>
+      <c r="B3"/>
+      <c r="C3"/>
+    </row>
+    <row r="4">
       <c r="A4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+      <c r="B4"/>
+      <c r="C4"/>
+    </row>
+    <row r="5">
       <c r="A5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>180</v>
+      </c>
+      <c r="B5"/>
+      <c r="C5"/>
+    </row>
+    <row r="6">
       <c r="A6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>181</v>
+      </c>
+      <c r="B6"/>
+      <c r="C6"/>
+    </row>
+    <row r="7">
       <c r="A7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+        <v>182</v>
+      </c>
+      <c r="B7"/>
+      <c r="C7"/>
+    </row>
+    <row r="8">
       <c r="A8" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+        <v>183</v>
+      </c>
+      <c r="B8"/>
+      <c r="C8"/>
+    </row>
+    <row r="9">
       <c r="A9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+        <v>184</v>
+      </c>
+      <c r="B9"/>
+      <c r="C9"/>
+    </row>
+    <row r="10">
       <c r="A10" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+        <v>185</v>
+      </c>
+      <c r="B10"/>
+      <c r="C10"/>
+    </row>
+    <row r="11">
       <c r="A11" t="s">
-        <v>59</v>
+        <v>182</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
-      </c>
-      <c r="C11">
-        <v>200.8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+        <v>186</v>
+      </c>
+      <c r="C11" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+        <v>188</v>
+      </c>
+      <c r="B12"/>
+      <c r="C12"/>
+    </row>
+    <row r="13">
       <c r="A13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+        <v>189</v>
+      </c>
+      <c r="B13"/>
+      <c r="C13"/>
+    </row>
+    <row r="14">
       <c r="A14" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+        <v>190</v>
+      </c>
+      <c r="B14"/>
+      <c r="C14"/>
+    </row>
+    <row r="15">
       <c r="A15" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+        <v>191</v>
+      </c>
+      <c r="B15"/>
+      <c r="C15"/>
+    </row>
+    <row r="16">
       <c r="A16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+        <v>192</v>
+      </c>
+      <c r="B16"/>
+      <c r="C16"/>
+    </row>
+    <row r="17">
       <c r="A17" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+        <v>193</v>
+      </c>
+      <c r="B17"/>
+      <c r="C17"/>
+    </row>
+    <row r="18">
       <c r="A18" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+        <v>194</v>
+      </c>
+      <c r="B18"/>
+      <c r="C18"/>
+    </row>
+    <row r="19">
       <c r="A19" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+        <v>195</v>
+      </c>
+      <c r="B19"/>
+      <c r="C19"/>
+    </row>
+    <row r="20">
       <c r="A20" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+        <v>196</v>
+      </c>
+      <c r="B20"/>
+      <c r="C20"/>
+    </row>
+    <row r="21">
       <c r="A21" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+        <v>197</v>
+      </c>
+      <c r="B21"/>
+      <c r="C21"/>
+    </row>
+    <row r="22">
       <c r="A22" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+        <v>198</v>
+      </c>
+      <c r="B22"/>
+      <c r="C22"/>
+    </row>
+    <row r="23">
       <c r="A23" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+        <v>199</v>
+      </c>
+      <c r="B23"/>
+      <c r="C23"/>
+    </row>
+    <row r="24">
       <c r="A24" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+        <v>200</v>
+      </c>
+      <c r="B24"/>
+      <c r="C24"/>
+    </row>
+    <row r="25">
       <c r="A25" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+        <v>201</v>
+      </c>
+      <c r="B25"/>
+      <c r="C25"/>
+    </row>
+    <row r="26">
       <c r="A26" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+        <v>202</v>
+      </c>
+      <c r="B26"/>
+      <c r="C26"/>
+    </row>
+    <row r="27">
       <c r="A27" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+        <v>203</v>
+      </c>
+      <c r="B27"/>
+      <c r="C27"/>
+    </row>
+    <row r="28">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>204</v>
       </c>
       <c r="B28" t="s">
-        <v>90</v>
+        <v>205</v>
       </c>
       <c r="C28" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="29">
       <c r="A29" t="s">
-        <v>77</v>
+        <v>207</v>
       </c>
       <c r="B29" t="s">
-        <v>127</v>
+        <v>208</v>
       </c>
       <c r="C29" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="30">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>207</v>
       </c>
       <c r="B30" t="s">
-        <v>125</v>
+        <v>210</v>
       </c>
       <c r="C30" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="31">
       <c r="A31" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+        <v>212</v>
+      </c>
+      <c r="B31"/>
+      <c r="C31"/>
+    </row>
+    <row r="32">
       <c r="A32" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+        <v>213</v>
+      </c>
+      <c r="B32"/>
+      <c r="C32"/>
+    </row>
+    <row r="33">
       <c r="A33" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+        <v>214</v>
+      </c>
+      <c r="B33"/>
+      <c r="C33"/>
+    </row>
+    <row r="34">
       <c r="A34" t="s">
-        <v>81</v>
+        <v>215</v>
       </c>
       <c r="B34" t="s">
-        <v>87</v>
-      </c>
-      <c r="C34">
-        <v>200.7</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+        <v>216</v>
+      </c>
+      <c r="C34" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="35">
       <c r="A35" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+        <v>218</v>
+      </c>
+      <c r="B35"/>
+      <c r="C35"/>
+    </row>
+    <row r="36">
       <c r="A36" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+        <v>219</v>
+      </c>
+      <c r="B36"/>
+      <c r="C36"/>
+    </row>
+    <row r="37">
       <c r="A37" t="s">
-        <v>84</v>
+        <v>220</v>
       </c>
       <c r="B37" t="s">
-        <v>93</v>
+        <v>221</v>
       </c>
       <c r="C37" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="38">
       <c r="A38" t="s">
-        <v>85</v>
-      </c>
+        <v>223</v>
+      </c>
+      <c r="B38"/>
+      <c r="C38"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="32.5546875" customWidth="1"/>
+    <col min="1" max="1" width="32.5546875" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" s="2" t="s">
         <v>95</v>
       </c>
@@ -1877,12 +2075,12 @@
         <v>105</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" s="3" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" t="s">
         <v>97</v>
       </c>
@@ -1890,27 +2088,27 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="A4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5">
       <c r="A5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6">
       <c r="A6" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7">
       <c r="A7" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8">
       <c r="A8" t="s">
         <v>102</v>
       </c>
@@ -1920,19 +2118,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="20.33203125" customWidth="1"/>
-    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="17" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" t="s">
         <v>114</v>
       </c>
@@ -1943,29 +2142,29 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" t="s">
         <v>106</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="n">
         <v>200.7</v>
       </c>
       <c r="C2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" t="s">
         <v>106</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="n">
         <v>200.8</v>
       </c>
       <c r="C3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="A4" t="s">
         <v>107</v>
       </c>
@@ -1976,7 +2175,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5">
       <c r="A5" t="s">
         <v>107</v>
       </c>
@@ -1987,7 +2186,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6">
       <c r="A6" t="s">
         <v>113</v>
       </c>
@@ -1998,7 +2197,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7">
       <c r="B7" t="s">
         <v>112</v>
       </c>
@@ -2008,20 +2207,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="24.44140625" customWidth="1"/>
-    <col min="2" max="2" width="22.88671875" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="22.88671875" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" t="s">
         <v>118</v>
       </c>
@@ -2035,7 +2235,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" t="s">
         <v>116</v>
       </c>
@@ -2049,35 +2249,35 @@
         <v>122</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" t="s">
         <v>116</v>
       </c>
       <c r="B3" t="s">
         <v>120</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>200.7</v>
       </c>
       <c r="D3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="A4" t="s">
         <v>116</v>
       </c>
       <c r="B4" t="s">
         <v>120</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>200.8</v>
       </c>
       <c r="D4" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5">
       <c r="A5" t="s">
         <v>117</v>
       </c>
@@ -2091,7 +2291,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6">
       <c r="A6" t="s">
         <v>116</v>
       </c>
@@ -2105,7 +2305,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7">
       <c r="A7" t="s">
         <v>116</v>
       </c>
@@ -2119,7 +2319,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8">
       <c r="A8" t="s">
         <v>116</v>
       </c>
@@ -2133,13 +2333,13 @@
         <v>90</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="18">
       <c r="B18" t="s">
         <v>45</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>